<commit_message>
completed implementation of stage 3.3 of boq logic
</commit_message>
<xml_diff>
--- a/besmm4_generated.xlsx
+++ b/besmm4_generated.xlsx
@@ -4,14 +4,14 @@
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="BESMM4 BoQ" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="_audit" sheetId="2" state="hidden" r:id="rId2"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
 </workbook>
 </file>
 
@@ -19,30 +19,57 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="#,##0.##"/>
-    <numFmt numFmtId="165" formatCode="&quot;₦&quot;#,##0.00"/>
+    <numFmt numFmtId="165" formatCode="\₦#,##0.00"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
+      <charset val="1"/>
       <family val="2"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font/>
-    <font>
-      <b val="1"/>
     </font>
     <font>
+      <name val="Arial"/>
+      <family val="0"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <family val="0"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <family val="0"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Cambria"/>
+      <charset val="1"/>
+      <family val="0"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Cambria"/>
+      <charset val="1"/>
+      <family val="0"/>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Cambria"/>
+      <charset val="1"/>
+      <family val="0"/>
       <b val="1"/>
       <sz val="12"/>
     </font>
     <font>
+      <name val="Cambria"/>
+      <charset val="1"/>
+      <family val="0"/>
       <i val="1"/>
       <sz val="11"/>
-    </font>
-    <font>
-      <i val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -53,7 +80,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -61,36 +88,75 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border/>
   </borders>
-  <cellStyleXfs count="3">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="1"/>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="1"/>
+  <cellStyleXfs count="8">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="43" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="41" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="44" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" applyAlignment="1">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" applyAlignment="1">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="7">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
-      <alignment horizontal="right"/>
+  <cellXfs count="14">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left"/>
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="21">
+      <alignment horizontal="right" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="20">
+      <alignment horizontal="right" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="21">
+      <alignment horizontal="right" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="bottom"/>
     </xf>
   </cellXfs>
-  <cellStyles count="3">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
-    <cellStyle name="qty_fmt" xfId="1" hidden="0"/>
-    <cellStyle name="currency_fmt" xfId="2" hidden="0"/>
+  <cellStyles count="8">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Comma" xfId="1" builtinId="3"/>
+    <cellStyle name="Comma [0]" xfId="2" builtinId="6"/>
+    <cellStyle name="Currency" xfId="3" builtinId="4"/>
+    <cellStyle name="Currency [0]" xfId="4" builtinId="7"/>
+    <cellStyle name="Percent" xfId="5" builtinId="5"/>
+    <cellStyle name="currency_fmt" xfId="6"/>
+    <cellStyle name="qty_fmt" xfId="7"/>
   </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="00000000"/>
@@ -447,84 +513,84 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
+  <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="0"/>
   </sheetPr>
   <dimension ref="A1:F77"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.54296875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" style="7" min="1" max="1"/>
+    <col width="60" customWidth="1" style="7" min="2" max="2"/>
+    <col width="10" customWidth="1" style="7" min="3" max="3"/>
+    <col width="14" customWidth="1" style="7" min="4" max="4"/>
+    <col width="16" customWidth="1" style="7" min="5" max="5"/>
+    <col width="18" customWidth="1" style="7" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="15" customHeight="1" s="8">
+      <c r="A1" s="9" t="inlineStr">
         <is>
           <t>Item Code</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="9" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="9" t="inlineStr">
         <is>
           <t>Unit</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="9" t="inlineStr">
         <is>
           <t>Quantity</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="9" t="inlineStr">
         <is>
           <t>Rate (₦)</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="9" t="inlineStr">
         <is>
           <t>Amount (₦)</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+    <row r="2" ht="15" customHeight="1" s="8">
+      <c r="A2" s="10" t="inlineStr">
         <is>
           <t>2.0 Substructure</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+    <row r="3" ht="15" customHeight="1" s="8">
+      <c r="A3" s="11" t="inlineStr">
         <is>
           <t>2.1 Excavating &amp; Filling</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
+    <row r="4" ht="15" customHeight="1" s="8">
+      <c r="A4" s="7" t="inlineStr">
         <is>
           <t>2.1.1</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr">
         <is>
           <t>Bulk excavation</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="7" t="inlineStr">
         <is>
           <t>m3</t>
         </is>
       </c>
-      <c r="D4" s="4" t="n">
+      <c r="D4" s="12" t="n">
         <v>0</v>
       </c>
       <c r="E4" s="5" t="n">
@@ -534,23 +600,23 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
+    <row r="5" ht="15" customHeight="1" s="8">
+      <c r="A5" s="7" t="inlineStr">
         <is>
           <t>2.1.2</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr">
         <is>
           <t>Foundation excavation</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="7" t="inlineStr">
         <is>
           <t>m3</t>
         </is>
       </c>
-      <c r="D5" s="4" t="n">
+      <c r="D5" s="12" t="n">
         <v>0</v>
       </c>
       <c r="E5" s="5" t="n">
@@ -560,23 +626,23 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
+    <row r="6" ht="15" customHeight="1" s="8">
+      <c r="A6" s="7" t="inlineStr">
         <is>
           <t>2.1.3</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr">
         <is>
           <t>Disposal off-site of excavated material</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="7" t="inlineStr">
         <is>
           <t>m3</t>
         </is>
       </c>
-      <c r="D6" s="4" t="n">
+      <c r="D6" s="12" t="n">
         <v>0</v>
       </c>
       <c r="E6" s="5" t="n">
@@ -586,23 +652,23 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
+    <row r="7" ht="15" customHeight="1" s="8">
+      <c r="A7" s="7" t="inlineStr">
         <is>
           <t>2.1.4</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr">
         <is>
           <t>Filling obtained from excavated material</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="7" t="inlineStr">
         <is>
           <t>m3</t>
         </is>
       </c>
-      <c r="D7" s="4" t="n">
+      <c r="D7" s="12" t="n">
         <v>0</v>
       </c>
       <c r="E7" s="5" t="n">
@@ -612,8 +678,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="6" t="inlineStr">
+    <row r="8" ht="15" customHeight="1" s="8">
+      <c r="A8" s="13" t="inlineStr">
         <is>
           <t>To Collection (2.1 Excavating &amp; Filling)</t>
         </is>
@@ -623,30 +689,30 @@
       </c>
     </row>
     <row r="9"/>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
+    <row r="10" ht="15" customHeight="1" s="8">
+      <c r="A10" s="11" t="inlineStr">
         <is>
           <t>2.2 Concrete Work</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
+    <row r="11" ht="15" customHeight="1" s="8">
+      <c r="A11" s="7" t="inlineStr">
         <is>
           <t>2.2.1</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="7" t="inlineStr">
         <is>
           <t>Blinding concrete</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C11" s="7" t="inlineStr">
         <is>
           <t>m3</t>
         </is>
       </c>
-      <c r="D11" s="4" t="n">
+      <c r="D11" s="12" t="n">
         <v>0</v>
       </c>
       <c r="E11" s="5" t="n">
@@ -656,23 +722,23 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
+    <row r="12" ht="15" customHeight="1" s="8">
+      <c r="A12" s="7" t="inlineStr">
         <is>
           <t>2.2.2</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="7" t="inlineStr">
         <is>
           <t>Reinforced concrete in foundations</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C12" s="7" t="inlineStr">
         <is>
           <t>m3</t>
         </is>
       </c>
-      <c r="D12" s="4" t="n">
+      <c r="D12" s="12" t="n">
         <v>0</v>
       </c>
       <c r="E12" s="5" t="n">
@@ -682,23 +748,23 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
+    <row r="13" ht="15" customHeight="1" s="8">
+      <c r="A13" s="7" t="inlineStr">
         <is>
           <t>2.2.3</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B13" s="7" t="inlineStr">
         <is>
           <t>Reinforced concrete ground floor slab</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C13" s="7" t="inlineStr">
         <is>
           <t>m2</t>
         </is>
       </c>
-      <c r="D13" s="4" t="n">
+      <c r="D13" s="12" t="n">
         <v>0</v>
       </c>
       <c r="E13" s="5" t="n">
@@ -708,8 +774,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="6" t="inlineStr">
+    <row r="14" ht="15" customHeight="1" s="8">
+      <c r="A14" s="13" t="inlineStr">
         <is>
           <t>To Collection (2.2 Concrete Work)</t>
         </is>
@@ -719,30 +785,30 @@
       </c>
     </row>
     <row r="15"/>
-    <row r="16">
-      <c r="A16" s="3" t="inlineStr">
+    <row r="16" ht="15" customHeight="1" s="8">
+      <c r="A16" s="11" t="inlineStr">
         <is>
           <t>2.3 Damp Proofing &amp; Membranes</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
+    <row r="17" ht="15" customHeight="1" s="8">
+      <c r="A17" s="7" t="inlineStr">
         <is>
           <t>2.3.1</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B17" s="7" t="inlineStr">
         <is>
           <t>Damp proof membrane</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C17" s="7" t="inlineStr">
         <is>
           <t>m2</t>
         </is>
       </c>
-      <c r="D17" s="4" t="n">
+      <c r="D17" s="12" t="n">
         <v>0</v>
       </c>
       <c r="E17" s="5" t="n">
@@ -752,8 +818,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="6" t="inlineStr">
+    <row r="18" ht="15" customHeight="1" s="8">
+      <c r="A18" s="13" t="inlineStr">
         <is>
           <t>To Collection (2.3 Damp Proofing &amp; Membranes)</t>
         </is>
@@ -763,37 +829,37 @@
       </c>
     </row>
     <row r="19"/>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
+    <row r="20" ht="15" customHeight="1" s="8">
+      <c r="A20" s="10" t="inlineStr">
         <is>
           <t>3.0 Superstructure</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="3" t="inlineStr">
+    <row r="21" ht="15" customHeight="1" s="8">
+      <c r="A21" s="11" t="inlineStr">
         <is>
           <t>3.1 Masonry / Blockwork</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
+    <row r="22" ht="15" customHeight="1" s="8">
+      <c r="A22" s="7" t="inlineStr">
         <is>
           <t>3.1.1</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B22" s="7" t="inlineStr">
         <is>
           <t>Blockwork 225mm thick in cement mortar</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C22" s="7" t="inlineStr">
         <is>
           <t>m2</t>
         </is>
       </c>
-      <c r="D22" s="4" t="n">
+      <c r="D22" s="12" t="n">
         <v>0</v>
       </c>
       <c r="E22" s="5" t="n">
@@ -803,23 +869,23 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
+    <row r="23" ht="15" customHeight="1" s="8">
+      <c r="A23" s="7" t="inlineStr">
         <is>
           <t>3.1.2</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B23" s="7" t="inlineStr">
         <is>
           <t>Partition walls</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C23" s="7" t="inlineStr">
         <is>
           <t>m2</t>
         </is>
       </c>
-      <c r="D23" s="4" t="n">
+      <c r="D23" s="12" t="n">
         <v>0</v>
       </c>
       <c r="E23" s="5" t="n">
@@ -829,8 +895,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="6" t="inlineStr">
+    <row r="24" ht="15" customHeight="1" s="8">
+      <c r="A24" s="13" t="inlineStr">
         <is>
           <t>To Collection (3.1 Masonry / Blockwork)</t>
         </is>
@@ -840,30 +906,30 @@
       </c>
     </row>
     <row r="25"/>
-    <row r="26">
-      <c r="A26" s="3" t="inlineStr">
+    <row r="26" ht="15" customHeight="1" s="8">
+      <c r="A26" s="11" t="inlineStr">
         <is>
           <t>3.2 Structural Concrete &amp; Steel</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
+    <row r="27" ht="15" customHeight="1" s="8">
+      <c r="A27" s="7" t="inlineStr">
         <is>
           <t>3.2.1</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B27" s="7" t="inlineStr">
         <is>
           <t>Reinforced concrete columns</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C27" s="7" t="inlineStr">
         <is>
           <t>m3</t>
         </is>
       </c>
-      <c r="D27" s="4" t="n">
+      <c r="D27" s="12" t="n">
         <v>0</v>
       </c>
       <c r="E27" s="5" t="n">
@@ -873,23 +939,23 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
+    <row r="28" ht="15" customHeight="1" s="8">
+      <c r="A28" s="7" t="inlineStr">
         <is>
           <t>3.2.2</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="B28" s="7" t="inlineStr">
         <is>
           <t>Structural steelwork</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C28" s="7" t="inlineStr">
         <is>
           <t>t</t>
         </is>
       </c>
-      <c r="D28" s="4" t="n">
+      <c r="D28" s="12" t="n">
         <v>0</v>
       </c>
       <c r="E28" s="5" t="n">
@@ -899,8 +965,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="6" t="inlineStr">
+    <row r="29" ht="15" customHeight="1" s="8">
+      <c r="A29" s="13" t="inlineStr">
         <is>
           <t>To Collection (3.2 Structural Concrete &amp; Steel)</t>
         </is>
@@ -910,30 +976,30 @@
       </c>
     </row>
     <row r="30"/>
-    <row r="31">
-      <c r="A31" s="3" t="inlineStr">
+    <row r="31" ht="15" customHeight="1" s="8">
+      <c r="A31" s="11" t="inlineStr">
         <is>
           <t>3.3 Openings</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
+    <row r="32" ht="15" customHeight="1" s="8">
+      <c r="A32" s="7" t="inlineStr">
         <is>
           <t>3.3.1</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="B32" s="7" t="inlineStr">
         <is>
           <t>Doors (supply &amp; fix)</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
+      <c r="C32" s="7" t="inlineStr">
         <is>
           <t>No.</t>
         </is>
       </c>
-      <c r="D32" s="4" t="n">
+      <c r="D32" s="12" t="n">
         <v>12</v>
       </c>
       <c r="E32" s="5" t="n">
@@ -943,23 +1009,23 @@
         <v>540000</v>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
+    <row r="33" ht="15" customHeight="1" s="8">
+      <c r="A33" s="7" t="inlineStr">
         <is>
           <t>3.3.2</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
+      <c r="B33" s="7" t="inlineStr">
         <is>
           <t>Windows (supply &amp; fix)</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="C33" s="7" t="inlineStr">
         <is>
           <t>No.</t>
         </is>
       </c>
-      <c r="D33" s="4" t="n">
+      <c r="D33" s="12" t="n">
         <v>19</v>
       </c>
       <c r="E33" s="5" t="n">
@@ -969,8 +1035,8 @@
         <v>760000</v>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="6" t="inlineStr">
+    <row r="34" ht="15" customHeight="1" s="8">
+      <c r="A34" s="13" t="inlineStr">
         <is>
           <t>To Collection (3.3 Openings)</t>
         </is>
@@ -980,37 +1046,37 @@
       </c>
     </row>
     <row r="35"/>
-    <row r="36">
-      <c r="A36" s="2" t="inlineStr">
+    <row r="36" ht="15" customHeight="1" s="8">
+      <c r="A36" s="10" t="inlineStr">
         <is>
           <t>4.0 Finishes</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="3" t="inlineStr">
+    <row r="37" ht="15" customHeight="1" s="8">
+      <c r="A37" s="11" t="inlineStr">
         <is>
           <t>4.1 Internal Finishes</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
+    <row r="38" ht="15" customHeight="1" s="8">
+      <c r="A38" s="7" t="inlineStr">
         <is>
           <t>4.1.1</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr">
+      <c r="B38" s="7" t="inlineStr">
         <is>
           <t>Internal plastering 12mm</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
+      <c r="C38" s="7" t="inlineStr">
         <is>
           <t>m2</t>
         </is>
       </c>
-      <c r="D38" s="4" t="n">
+      <c r="D38" s="12" t="n">
         <v>0</v>
       </c>
       <c r="E38" s="5" t="n">
@@ -1020,23 +1086,23 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
+    <row r="39" ht="15" customHeight="1" s="8">
+      <c r="A39" s="7" t="inlineStr">
         <is>
           <t>4.1.2</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr">
+      <c r="B39" s="7" t="inlineStr">
         <is>
           <t>Floor tiling (ceramic)</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr">
+      <c r="C39" s="7" t="inlineStr">
         <is>
           <t>m2</t>
         </is>
       </c>
-      <c r="D39" s="4" t="n">
+      <c r="D39" s="12" t="n">
         <v>0</v>
       </c>
       <c r="E39" s="5" t="n">
@@ -1046,23 +1112,23 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
+    <row r="40" ht="15" customHeight="1" s="8">
+      <c r="A40" s="7" t="inlineStr">
         <is>
           <t>4.1.3</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr">
+      <c r="B40" s="7" t="inlineStr">
         <is>
           <t>Skirting (supply &amp; fix)</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr">
+      <c r="C40" s="7" t="inlineStr">
         <is>
           <t>m</t>
         </is>
       </c>
-      <c r="D40" s="4" t="n">
+      <c r="D40" s="12" t="n">
         <v>0</v>
       </c>
       <c r="E40" s="5" t="n">
@@ -1072,23 +1138,23 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
+    <row r="41" ht="15" customHeight="1" s="8">
+      <c r="A41" s="7" t="inlineStr">
         <is>
           <t>4.1.4</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr">
+      <c r="B41" s="7" t="inlineStr">
         <is>
           <t>Ceiling finishes (gypsum/POP/PVC)</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr">
+      <c r="C41" s="7" t="inlineStr">
         <is>
           <t>m2</t>
         </is>
       </c>
-      <c r="D41" s="4" t="n">
+      <c r="D41" s="12" t="n">
         <v>0</v>
       </c>
       <c r="E41" s="5" t="n">
@@ -1098,23 +1164,23 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
+    <row r="42" ht="15" customHeight="1" s="8">
+      <c r="A42" s="7" t="inlineStr">
         <is>
           <t>4.1.5</t>
         </is>
       </c>
-      <c r="B42" t="inlineStr">
+      <c r="B42" s="7" t="inlineStr">
         <is>
           <t>Painting to walls (2 coats)</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr">
+      <c r="C42" s="7" t="inlineStr">
         <is>
           <t>m2</t>
         </is>
       </c>
-      <c r="D42" s="4" t="n">
+      <c r="D42" s="12" t="n">
         <v>0</v>
       </c>
       <c r="E42" s="5" t="n">
@@ -1124,8 +1190,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="6" t="inlineStr">
+    <row r="43" ht="15" customHeight="1" s="8">
+      <c r="A43" s="13" t="inlineStr">
         <is>
           <t>To Collection (4.1 Internal Finishes)</t>
         </is>
@@ -1135,37 +1201,37 @@
       </c>
     </row>
     <row r="44"/>
-    <row r="45">
-      <c r="A45" s="2" t="inlineStr">
+    <row r="45" ht="15" customHeight="1" s="8">
+      <c r="A45" s="10" t="inlineStr">
         <is>
           <t>5.0 Fittings &amp; Fixtures</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="3" t="inlineStr">
+    <row r="46" ht="15" customHeight="1" s="8">
+      <c r="A46" s="11" t="inlineStr">
         <is>
           <t>5.1 Fittings &amp; Fixtures</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
+    <row r="47" ht="15" customHeight="1" s="8">
+      <c r="A47" s="7" t="inlineStr">
         <is>
           <t>5.1.1</t>
         </is>
       </c>
-      <c r="B47" t="inlineStr">
+      <c r="B47" s="7" t="inlineStr">
         <is>
           <t>Sanitary fittings (WC, basin, etc.)</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr">
+      <c r="C47" s="7" t="inlineStr">
         <is>
           <t>No.</t>
         </is>
       </c>
-      <c r="D47" s="4" t="n">
+      <c r="D47" s="12" t="n">
         <v>0</v>
       </c>
       <c r="E47" s="5" t="n">
@@ -1175,23 +1241,23 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
+    <row r="48" ht="15" customHeight="1" s="8">
+      <c r="A48" s="7" t="inlineStr">
         <is>
           <t>5.1.2</t>
         </is>
       </c>
-      <c r="B48" t="inlineStr">
+      <c r="B48" s="7" t="inlineStr">
         <is>
           <t>Kitchen fittings (complete)</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr">
+      <c r="C48" s="7" t="inlineStr">
         <is>
           <t>No.</t>
         </is>
       </c>
-      <c r="D48" s="4" t="n">
+      <c r="D48" s="12" t="n">
         <v>0</v>
       </c>
       <c r="E48" s="5" t="n">
@@ -1201,23 +1267,23 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
+    <row r="49" ht="15" customHeight="1" s="8">
+      <c r="A49" s="7" t="inlineStr">
         <is>
           <t>5.1.3</t>
         </is>
       </c>
-      <c r="B49" t="inlineStr">
+      <c r="B49" s="7" t="inlineStr">
         <is>
           <t>Wardrobes (supply &amp; fix)</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
+      <c r="C49" s="7" t="inlineStr">
         <is>
           <t>No.</t>
         </is>
       </c>
-      <c r="D49" s="4" t="n">
+      <c r="D49" s="12" t="n">
         <v>0</v>
       </c>
       <c r="E49" s="5" t="n">
@@ -1227,8 +1293,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" s="6" t="inlineStr">
+    <row r="50" ht="15" customHeight="1" s="8">
+      <c r="A50" s="13" t="inlineStr">
         <is>
           <t>To Collection (5.1 Fittings &amp; Fixtures)</t>
         </is>
@@ -1238,37 +1304,37 @@
       </c>
     </row>
     <row r="51"/>
-    <row r="52">
-      <c r="A52" s="2" t="inlineStr">
+    <row r="52" ht="15" customHeight="1" s="8">
+      <c r="A52" s="10" t="inlineStr">
         <is>
           <t>6.0 Mechanical &amp; Electrical Works</t>
         </is>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" s="3" t="inlineStr">
+    <row r="53" ht="15" customHeight="1" s="8">
+      <c r="A53" s="11" t="inlineStr">
         <is>
           <t>6.1 Mechanical Services</t>
         </is>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
+    <row r="54" ht="15" customHeight="1" s="8">
+      <c r="A54" s="7" t="inlineStr">
         <is>
           <t>6.1.1</t>
         </is>
       </c>
-      <c r="B54" t="inlineStr">
+      <c r="B54" s="7" t="inlineStr">
         <is>
           <t>Plumbing fittings (points)</t>
         </is>
       </c>
-      <c r="C54" t="inlineStr">
+      <c r="C54" s="7" t="inlineStr">
         <is>
           <t>No.</t>
         </is>
       </c>
-      <c r="D54" s="4" t="n">
+      <c r="D54" s="12" t="n">
         <v>0</v>
       </c>
       <c r="E54" s="5" t="n">
@@ -1278,23 +1344,23 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
+    <row r="55" ht="15" customHeight="1" s="8">
+      <c r="A55" s="7" t="inlineStr">
         <is>
           <t>6.1.2</t>
         </is>
       </c>
-      <c r="B55" t="inlineStr">
+      <c r="B55" s="7" t="inlineStr">
         <is>
           <t>HVAC system (per system)</t>
         </is>
       </c>
-      <c r="C55" t="inlineStr">
+      <c r="C55" s="7" t="inlineStr">
         <is>
           <t>No.</t>
         </is>
       </c>
-      <c r="D55" s="4" t="n">
+      <c r="D55" s="12" t="n">
         <v>0</v>
       </c>
       <c r="E55" s="5" t="n">
@@ -1304,8 +1370,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" s="6" t="inlineStr">
+    <row r="56" ht="15" customHeight="1" s="8">
+      <c r="A56" s="13" t="inlineStr">
         <is>
           <t>To Collection (6.1 Mechanical Services)</t>
         </is>
@@ -1315,30 +1381,30 @@
       </c>
     </row>
     <row r="57"/>
-    <row r="58">
-      <c r="A58" s="3" t="inlineStr">
+    <row r="58" ht="15" customHeight="1" s="8">
+      <c r="A58" s="11" t="inlineStr">
         <is>
           <t>6.2 Electrical Services</t>
         </is>
       </c>
     </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
+    <row r="59" ht="15" customHeight="1" s="8">
+      <c r="A59" s="7" t="inlineStr">
         <is>
           <t>6.2.1</t>
         </is>
       </c>
-      <c r="B59" t="inlineStr">
+      <c r="B59" s="7" t="inlineStr">
         <is>
           <t>Lighting fittings</t>
         </is>
       </c>
-      <c r="C59" t="inlineStr">
+      <c r="C59" s="7" t="inlineStr">
         <is>
           <t>No.</t>
         </is>
       </c>
-      <c r="D59" s="4" t="n">
+      <c r="D59" s="12" t="n">
         <v>0</v>
       </c>
       <c r="E59" s="5" t="n">
@@ -1348,23 +1414,23 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
+    <row r="60" ht="15" customHeight="1" s="8">
+      <c r="A60" s="7" t="inlineStr">
         <is>
           <t>6.2.2</t>
         </is>
       </c>
-      <c r="B60" t="inlineStr">
+      <c r="B60" s="7" t="inlineStr">
         <is>
           <t>Power points</t>
         </is>
       </c>
-      <c r="C60" t="inlineStr">
+      <c r="C60" s="7" t="inlineStr">
         <is>
           <t>No.</t>
         </is>
       </c>
-      <c r="D60" s="4" t="n">
+      <c r="D60" s="12" t="n">
         <v>0</v>
       </c>
       <c r="E60" s="5" t="n">
@@ -1374,23 +1440,23 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
+    <row r="61" ht="15" customHeight="1" s="8">
+      <c r="A61" s="7" t="inlineStr">
         <is>
           <t>6.2.3</t>
         </is>
       </c>
-      <c r="B61" t="inlineStr">
+      <c r="B61" s="7" t="inlineStr">
         <is>
           <t>CCTV</t>
         </is>
       </c>
-      <c r="C61" t="inlineStr">
+      <c r="C61" s="7" t="inlineStr">
         <is>
           <t>No.</t>
         </is>
       </c>
-      <c r="D61" s="4" t="n">
+      <c r="D61" s="12" t="n">
         <v>0</v>
       </c>
       <c r="E61" s="5" t="n">
@@ -1400,8 +1466,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62">
-      <c r="A62" s="6" t="inlineStr">
+    <row r="62" ht="15" customHeight="1" s="8">
+      <c r="A62" s="13" t="inlineStr">
         <is>
           <t>To Collection (6.2 Electrical Services)</t>
         </is>
@@ -1411,37 +1477,37 @@
       </c>
     </row>
     <row r="63"/>
-    <row r="64">
-      <c r="A64" s="2" t="inlineStr">
+    <row r="64" ht="15" customHeight="1" s="8">
+      <c r="A64" s="10" t="inlineStr">
         <is>
           <t>7.0 External Works</t>
         </is>
       </c>
     </row>
-    <row r="65">
-      <c r="A65" s="3" t="inlineStr">
+    <row r="65" ht="15" customHeight="1" s="8">
+      <c r="A65" s="11" t="inlineStr">
         <is>
           <t>7.1 External Works</t>
         </is>
       </c>
     </row>
-    <row r="66">
-      <c r="A66" t="inlineStr">
+    <row r="66" ht="15" customHeight="1" s="8">
+      <c r="A66" s="7" t="inlineStr">
         <is>
           <t>7.1.1</t>
         </is>
       </c>
-      <c r="B66" t="inlineStr">
+      <c r="B66" s="7" t="inlineStr">
         <is>
           <t>Paving</t>
         </is>
       </c>
-      <c r="C66" t="inlineStr">
+      <c r="C66" s="7" t="inlineStr">
         <is>
           <t>m2</t>
         </is>
       </c>
-      <c r="D66" s="4" t="n">
+      <c r="D66" s="12" t="n">
         <v>0</v>
       </c>
       <c r="E66" s="5" t="n">
@@ -1451,23 +1517,23 @@
         <v>0</v>
       </c>
     </row>
-    <row r="67">
-      <c r="A67" t="inlineStr">
+    <row r="67" ht="15" customHeight="1" s="8">
+      <c r="A67" s="7" t="inlineStr">
         <is>
           <t>7.1.2</t>
         </is>
       </c>
-      <c r="B67" t="inlineStr">
+      <c r="B67" s="7" t="inlineStr">
         <is>
           <t>Driveways</t>
         </is>
       </c>
-      <c r="C67" t="inlineStr">
+      <c r="C67" s="7" t="inlineStr">
         <is>
           <t>m2</t>
         </is>
       </c>
-      <c r="D67" s="4" t="n">
+      <c r="D67" s="12" t="n">
         <v>0</v>
       </c>
       <c r="E67" s="5" t="n">
@@ -1477,23 +1543,23 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68">
-      <c r="A68" t="inlineStr">
+    <row r="68" ht="15" customHeight="1" s="8">
+      <c r="A68" s="7" t="inlineStr">
         <is>
           <t>7.1.3</t>
         </is>
       </c>
-      <c r="B68" t="inlineStr">
+      <c r="B68" s="7" t="inlineStr">
         <is>
           <t>Landscaping</t>
         </is>
       </c>
-      <c r="C68" t="inlineStr">
+      <c r="C68" s="7" t="inlineStr">
         <is>
           <t>m2</t>
         </is>
       </c>
-      <c r="D68" s="4" t="n">
+      <c r="D68" s="12" t="n">
         <v>0</v>
       </c>
       <c r="E68" s="5" t="n">
@@ -1503,8 +1569,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69">
-      <c r="A69" s="6" t="inlineStr">
+    <row r="69" ht="15" customHeight="1" s="8">
+      <c r="A69" s="13" t="inlineStr">
         <is>
           <t>To Collection (7.1 External Works)</t>
         </is>
@@ -1514,37 +1580,37 @@
       </c>
     </row>
     <row r="70"/>
-    <row r="71">
-      <c r="A71" s="2" t="inlineStr">
+    <row r="71" ht="15" customHeight="1" s="8">
+      <c r="A71" s="10" t="inlineStr">
         <is>
           <t>8.0 Provisional &amp; Prime Cost Sums</t>
         </is>
       </c>
     </row>
-    <row r="72">
-      <c r="A72" s="3" t="inlineStr">
+    <row r="72" ht="15" customHeight="1" s="8">
+      <c r="A72" s="11" t="inlineStr">
         <is>
           <t>8.1 Provisional Sums</t>
         </is>
       </c>
     </row>
-    <row r="73">
-      <c r="A73" t="inlineStr">
+    <row r="73" ht="15" customHeight="1" s="8">
+      <c r="A73" s="7" t="inlineStr">
         <is>
           <t>8.1.1</t>
         </is>
       </c>
-      <c r="B73" t="inlineStr">
+      <c r="B73" s="7" t="inlineStr">
         <is>
           <t>Specialized works (PC sum)</t>
         </is>
       </c>
-      <c r="C73" t="inlineStr">
+      <c r="C73" s="7" t="inlineStr">
         <is>
           <t>item</t>
         </is>
       </c>
-      <c r="D73" s="4" t="n">
+      <c r="D73" s="12" t="n">
         <v>0</v>
       </c>
       <c r="E73" s="5" t="n">
@@ -1554,23 +1620,23 @@
         <v>0</v>
       </c>
     </row>
-    <row r="74">
-      <c r="A74" t="inlineStr">
+    <row r="74" ht="15" customHeight="1" s="8">
+      <c r="A74" s="7" t="inlineStr">
         <is>
           <t>8.1.2</t>
         </is>
       </c>
-      <c r="B74" t="inlineStr">
+      <c r="B74" s="7" t="inlineStr">
         <is>
           <t>Contingencies</t>
         </is>
       </c>
-      <c r="C74" t="inlineStr">
+      <c r="C74" s="7" t="inlineStr">
         <is>
           <t>item</t>
         </is>
       </c>
-      <c r="D74" s="4" t="n">
+      <c r="D74" s="12" t="n">
         <v>0</v>
       </c>
       <c r="E74" s="5" t="n">
@@ -1580,8 +1646,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75">
-      <c r="A75" s="6" t="inlineStr">
+    <row r="75" ht="15" customHeight="1" s="8">
+      <c r="A75" s="13" t="inlineStr">
         <is>
           <t>To Collection (8.1 Provisional Sums)</t>
         </is>
@@ -1591,8 +1657,8 @@
       </c>
     </row>
     <row r="76"/>
-    <row r="77">
-      <c r="A77" s="2" t="inlineStr">
+    <row r="77" ht="15" customHeight="1" s="8">
+      <c r="A77" s="10" t="inlineStr">
         <is>
           <t>GRAND TOTAL</t>
         </is>
@@ -1609,8 +1675,8 @@
     <mergeCell ref="A46:F46"/>
     <mergeCell ref="A24:E24"/>
     <mergeCell ref="A37:F37"/>
+    <mergeCell ref="A3:F3"/>
     <mergeCell ref="A26:F26"/>
-    <mergeCell ref="A3:F3"/>
     <mergeCell ref="A21:F21"/>
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A69:E69"/>
@@ -1636,7 +1702,9 @@
     <mergeCell ref="A45:F45"/>
     <mergeCell ref="A65:F65"/>
   </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
 </worksheet>
 </file>
 
@@ -2037,7 +2105,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>kitchen store D2 W5 W6:1; kitchen store D2 W5 W6:5; FOYER W4:1; bath children's bedroom D3 W4 W6:5</t>
+          <t>Handler error; fallback to parsed qty ('dict' object has no attribute 'confirmed')</t>
         </is>
       </c>
     </row>
@@ -2068,7 +2136,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>MAIN LIVING ent. D1 D4 W1:1; children's bedroom bath D3 D3 D4 D4 D4 W6:5; kitchen store D2 W5 W6:1; master's W2 W2 W3:1; FOYER W4:6; FOYER W4:5</t>
+          <t>Handler error; fallback to parsed qty ('dict' object has no attribute 'confirmed')</t>
         </is>
       </c>
     </row>

</xml_diff>